<commit_message>
-> Updated metrics and images. -> Added more matrices tests.
</commit_message>
<xml_diff>
--- a/docs/cacheBandit_metrics.xlsx
+++ b/docs/cacheBandit_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91988\Documents\Amruth\Files\Git\cacheBandit\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675385A6-149D-4854-8554-E40826A3A93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F943A65-7185-4BB2-83DA-98580442DB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C4CDEA3B-1686-49FD-8414-9D1FD93CDC23}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="83">
   <si>
     <t>Thread Count</t>
   </si>
@@ -267,6 +267,15 @@
   <si>
     <t>Correlation positive lim</t>
   </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>The reason for this is: Diagonal matrices are purely streaming in the case of SpMV, as there is no re-use of cache lines across warps. This leads to the absence of thrashing, resulting in the random part of the global policy negatively impacting the cache usage.</t>
+  </si>
+  <si>
+    <t>LRU</t>
+  </si>
 </sst>
 </file>
 
@@ -325,12 +334,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -343,8 +353,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -885,6 +893,709 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cache Efficiency</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$109</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>LRU</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$C$105:$U$105</c:f>
+              <c:strCache>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>bcsstk10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>bcsstk13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>bcsstk17</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>c8_mat11</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>cq9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>fv1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>kl02</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>lhr34c</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>pdb1HYS</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>psmigr_1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>wiki-Vote</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>p2p-Gnutella04</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>ca-HepTh</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>as-735</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>amazon0312</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$109:$U$109</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.6807113925229294E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.5780260442610121E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.3561006894340225E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.836952380952381</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.40653454740224959</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.22234762979683972</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.8917246713070378E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.10119047619047619</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.150157813444362E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14255890247539516</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.3030685161832703</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.39307622869439407</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6B79-45CA-A76D-2552527AE457}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$110</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CacheBandit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$C$105:$U$105</c:f>
+              <c:strCache>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>bcsstk10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>bcsstk13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>bcsstk17</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>c8_mat11</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>cq9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>fv1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>kl02</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>lhr34c</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>pdb1HYS</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>psmigr_1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>wiki-Vote</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>p2p-Gnutella04</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>ca-HepTh</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>as-735</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>amazon0312</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$110:$U$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.60267111853088484</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.2142629735752945</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.478890229191798E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.87425387982491043</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.4882075471698113</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.86495726495726499</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.21963824289405684</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7.5319926873857398E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.5786516853932584</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.62454697134445358</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6B79-45CA-A76D-2552527AE457}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1038553776"/>
+        <c:axId val="1038552336"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1038553776"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1600"/>
+                  <a:t>Mtrix</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1038552336"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1038552336"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Efficiency (normalized)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1038553776"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:minorUnit val="5.000000000000001E-2"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -3125,9 +3836,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$23:$R$23</c:f>
+              <c:f>Sheet1!$C$23:$U$23</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>bcsstk10</c:v>
                 </c:pt>
@@ -3175,16 +3886,19 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$26:$R$26</c:f>
+              <c:f>Sheet1!$C$26:$U$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -3232,6 +3946,9 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>47.625052543085324</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>34.353165863987456</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4337,7 +5054,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Baseline Cache Efficiency</c:v>
+                  <c:v>LRU</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4354,9 +5071,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$23:$R$23</c:f>
+              <c:f>Sheet1!$C$23:$U$23</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>bcsstk10</c:v>
                 </c:pt>
@@ -4404,16 +5121,19 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$27:$R$27</c:f>
+              <c:f>Sheet1!$C$27:$U$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -4461,6 +5181,9 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0.3030685161832703</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.39307622869439407</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4480,7 +5203,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>CacheBandit Cache Efficiency</c:v>
+                  <c:v>CacheBandit</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4497,9 +5220,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$23:$R$23</c:f>
+              <c:f>Sheet1!$C$23:$U$23</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>bcsstk10</c:v>
                 </c:pt>
@@ -4547,16 +5270,19 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$28:$R$28</c:f>
+              <c:f>Sheet1!$C$28:$U$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -4604,6 +5330,9 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0.5786516853932584</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.61038406266350664</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5069,9 +5798,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$105:$R$105</c:f>
+              <c:f>Sheet1!$C$105:$U$105</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>bcsstk10</c:v>
                 </c:pt>
@@ -5119,16 +5848,19 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>sinc15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Average</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$108:$R$108</c:f>
+              <c:f>Sheet1!$C$108:$U$108</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -5176,6 +5908,9 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>47.625052543085324</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>36.215861874989677</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6375,6 +7110,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1558269472"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6433,6 +7169,46 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -7295,6 +8071,509 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
   <cs:axisTitle>
@@ -11650,6 +12929,42 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>11043</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>30921</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>77304</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>132521</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D41E1EF9-4DBB-6BB0-7F49-FCAAEFA69685}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -11986,209 +13301,209 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:40" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
-      <c r="AD2" s="4"/>
-      <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
-      <c r="AH2" s="4"/>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="4"/>
-      <c r="AK2" s="4"/>
-      <c r="AL2" s="4"/>
-      <c r="AM2" s="4"/>
-      <c r="AN2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+      <c r="X2" s="5"/>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="5"/>
+      <c r="AA2" s="5"/>
+      <c r="AB2" s="5"/>
+      <c r="AC2" s="5"/>
+      <c r="AD2" s="5"/>
+      <c r="AE2" s="5"/>
+      <c r="AF2" s="5"/>
+      <c r="AG2" s="5"/>
+      <c r="AH2" s="5"/>
+      <c r="AI2" s="5"/>
+      <c r="AJ2" s="5"/>
+      <c r="AK2" s="5"/>
+      <c r="AL2" s="5"/>
+      <c r="AM2" s="5"/>
+      <c r="AN2" s="5"/>
     </row>
     <row r="3" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="4"/>
+      <c r="G3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
+      <c r="J3" s="4"/>
+      <c r="K3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3" t="s">
+      <c r="L3" s="4"/>
+      <c r="M3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3" t="s">
+      <c r="N3" s="4"/>
+      <c r="O3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3" t="s">
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3" t="s">
+      <c r="R3" s="4"/>
+      <c r="S3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3" t="s">
+      <c r="T3" s="4"/>
+      <c r="U3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3" t="s">
+      <c r="V3" s="4"/>
+      <c r="W3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3" t="s">
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="3" t="s">
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3" t="s">
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AD3" s="3"/>
-      <c r="AE3" s="3" t="s">
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3" t="s">
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3" t="s">
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AJ3" s="3"/>
-      <c r="AK3" s="3" t="s">
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AL3" s="3"/>
-      <c r="AM3" s="3" t="s">
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AN3" s="3"/>
+      <c r="AN3" s="4"/>
     </row>
     <row r="4" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
+      <c r="F4" s="4"/>
+      <c r="G4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3" t="s">
+      <c r="H4" s="4"/>
+      <c r="I4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="4"/>
+      <c r="K4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3" t="s">
+      <c r="L4" s="4"/>
+      <c r="M4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3" t="s">
+      <c r="N4" s="4"/>
+      <c r="O4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3" t="s">
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3" t="s">
+      <c r="R4" s="4"/>
+      <c r="S4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3" t="s">
+      <c r="T4" s="4"/>
+      <c r="U4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3" t="s">
+      <c r="V4" s="4"/>
+      <c r="W4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3" t="s">
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3" t="s">
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="3" t="s">
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AD4" s="3"/>
-      <c r="AE4" s="3" t="s">
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="3" t="s">
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AH4" s="3"/>
-      <c r="AI4" s="3" t="s">
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AJ4" s="3"/>
-      <c r="AK4" s="3" t="s">
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AL4" s="3"/>
-      <c r="AM4" s="3" t="s">
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AN4" s="3"/>
+      <c r="AN4" s="4"/>
     </row>
     <row r="5" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
@@ -14257,209 +15572,209 @@
       </c>
     </row>
     <row r="63" spans="2:40" x14ac:dyDescent="0.3">
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-      <c r="L63" s="5"/>
-      <c r="M63" s="5"/>
-      <c r="N63" s="5"/>
-      <c r="O63" s="5"/>
-      <c r="P63" s="5"/>
-      <c r="Q63" s="5"/>
-      <c r="R63" s="5"/>
-      <c r="S63" s="5"/>
-      <c r="T63" s="5"/>
-      <c r="U63" s="5"/>
-      <c r="V63" s="5"/>
-      <c r="W63" s="5"/>
-      <c r="X63" s="5"/>
-      <c r="Y63" s="5"/>
-      <c r="Z63" s="5"/>
-      <c r="AA63" s="5"/>
-      <c r="AB63" s="5"/>
-      <c r="AC63" s="5"/>
-      <c r="AD63" s="5"/>
-      <c r="AE63" s="5"/>
-      <c r="AF63" s="5"/>
-      <c r="AG63" s="5"/>
-      <c r="AH63" s="5"/>
-      <c r="AI63" s="5"/>
-      <c r="AJ63" s="5"/>
-      <c r="AK63" s="5"/>
-      <c r="AL63" s="5"/>
-      <c r="AM63" s="5"/>
-      <c r="AN63" s="5"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6"/>
+      <c r="K63" s="6"/>
+      <c r="L63" s="6"/>
+      <c r="M63" s="6"/>
+      <c r="N63" s="6"/>
+      <c r="O63" s="6"/>
+      <c r="P63" s="6"/>
+      <c r="Q63" s="6"/>
+      <c r="R63" s="6"/>
+      <c r="S63" s="6"/>
+      <c r="T63" s="6"/>
+      <c r="U63" s="6"/>
+      <c r="V63" s="6"/>
+      <c r="W63" s="6"/>
+      <c r="X63" s="6"/>
+      <c r="Y63" s="6"/>
+      <c r="Z63" s="6"/>
+      <c r="AA63" s="6"/>
+      <c r="AB63" s="6"/>
+      <c r="AC63" s="6"/>
+      <c r="AD63" s="6"/>
+      <c r="AE63" s="6"/>
+      <c r="AF63" s="6"/>
+      <c r="AG63" s="6"/>
+      <c r="AH63" s="6"/>
+      <c r="AI63" s="6"/>
+      <c r="AJ63" s="6"/>
+      <c r="AK63" s="6"/>
+      <c r="AL63" s="6"/>
+      <c r="AM63" s="6"/>
+      <c r="AN63" s="6"/>
     </row>
     <row r="64" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>27</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3" t="s">
+      <c r="D64" s="4"/>
+      <c r="E64" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3" t="s">
+      <c r="F64" s="4"/>
+      <c r="G64" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H64" s="3"/>
-      <c r="I64" s="3" t="s">
+      <c r="H64" s="4"/>
+      <c r="I64" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J64" s="3"/>
-      <c r="K64" s="3" t="s">
+      <c r="J64" s="4"/>
+      <c r="K64" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="L64" s="3"/>
-      <c r="M64" s="3" t="s">
+      <c r="L64" s="4"/>
+      <c r="M64" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N64" s="3"/>
-      <c r="O64" s="3" t="s">
+      <c r="N64" s="4"/>
+      <c r="O64" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="P64" s="3"/>
-      <c r="Q64" s="3" t="s">
+      <c r="P64" s="4"/>
+      <c r="Q64" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R64" s="3"/>
-      <c r="S64" s="3" t="s">
+      <c r="R64" s="4"/>
+      <c r="S64" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="T64" s="3"/>
-      <c r="U64" s="3" t="s">
+      <c r="T64" s="4"/>
+      <c r="U64" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="V64" s="3"/>
-      <c r="W64" s="3" t="s">
+      <c r="V64" s="4"/>
+      <c r="W64" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="X64" s="3"/>
-      <c r="Y64" s="3" t="s">
+      <c r="X64" s="4"/>
+      <c r="Y64" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="Z64" s="3"/>
-      <c r="AA64" s="3" t="s">
+      <c r="Z64" s="4"/>
+      <c r="AA64" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AB64" s="3"/>
-      <c r="AC64" s="3" t="s">
+      <c r="AB64" s="4"/>
+      <c r="AC64" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AD64" s="3"/>
-      <c r="AE64" s="3" t="s">
+      <c r="AD64" s="4"/>
+      <c r="AE64" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AF64" s="3"/>
-      <c r="AG64" s="3" t="s">
+      <c r="AF64" s="4"/>
+      <c r="AG64" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AH64" s="3"/>
-      <c r="AI64" s="3" t="s">
+      <c r="AH64" s="4"/>
+      <c r="AI64" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AJ64" s="3"/>
-      <c r="AK64" s="3" t="s">
+      <c r="AJ64" s="4"/>
+      <c r="AK64" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AL64" s="3"/>
-      <c r="AM64" s="3" t="s">
+      <c r="AL64" s="4"/>
+      <c r="AM64" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AN64" s="3"/>
+      <c r="AN64" s="4"/>
     </row>
     <row r="65" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>26</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3" t="s">
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F65" s="3"/>
-      <c r="G65" s="3" t="s">
+      <c r="F65" s="4"/>
+      <c r="G65" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H65" s="3"/>
-      <c r="I65" s="3" t="s">
+      <c r="H65" s="4"/>
+      <c r="I65" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J65" s="3"/>
-      <c r="K65" s="3" t="s">
+      <c r="J65" s="4"/>
+      <c r="K65" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L65" s="3"/>
-      <c r="M65" s="3" t="s">
+      <c r="L65" s="4"/>
+      <c r="M65" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N65" s="3"/>
-      <c r="O65" s="3" t="s">
+      <c r="N65" s="4"/>
+      <c r="O65" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P65" s="3"/>
-      <c r="Q65" s="3" t="s">
+      <c r="P65" s="4"/>
+      <c r="Q65" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="R65" s="3"/>
-      <c r="S65" s="3" t="s">
+      <c r="R65" s="4"/>
+      <c r="S65" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T65" s="3"/>
-      <c r="U65" s="3" t="s">
+      <c r="T65" s="4"/>
+      <c r="U65" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V65" s="3"/>
-      <c r="W65" s="3" t="s">
+      <c r="V65" s="4"/>
+      <c r="W65" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="X65" s="3"/>
-      <c r="Y65" s="3" t="s">
+      <c r="X65" s="4"/>
+      <c r="Y65" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Z65" s="3"/>
-      <c r="AA65" s="3" t="s">
+      <c r="Z65" s="4"/>
+      <c r="AA65" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AB65" s="3"/>
-      <c r="AC65" s="3" t="s">
+      <c r="AB65" s="4"/>
+      <c r="AC65" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AD65" s="3"/>
-      <c r="AE65" s="3" t="s">
+      <c r="AD65" s="4"/>
+      <c r="AE65" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AF65" s="3"/>
-      <c r="AG65" s="3" t="s">
+      <c r="AF65" s="4"/>
+      <c r="AG65" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AH65" s="3"/>
-      <c r="AI65" s="3" t="s">
+      <c r="AH65" s="4"/>
+      <c r="AI65" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AJ65" s="3"/>
-      <c r="AK65" s="3" t="s">
+      <c r="AJ65" s="4"/>
+      <c r="AK65" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AL65" s="3"/>
-      <c r="AM65" s="3" t="s">
+      <c r="AL65" s="4"/>
+      <c r="AM65" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AN65" s="3"/>
+      <c r="AN65" s="4"/>
     </row>
     <row r="66" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
@@ -16615,213 +17930,213 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CEFDD9D-FDB3-41CB-A695-1350C2A9CE69}">
-  <dimension ref="B2:AN187"/>
+  <dimension ref="B2:AN188"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="2:40" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
-      <c r="AD2" s="4"/>
-      <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
-      <c r="AH2" s="4"/>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="4"/>
-      <c r="AK2" s="4"/>
-      <c r="AL2" s="4"/>
-      <c r="AM2" s="4"/>
-      <c r="AN2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+      <c r="X2" s="5"/>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="5"/>
+      <c r="AA2" s="5"/>
+      <c r="AB2" s="5"/>
+      <c r="AC2" s="5"/>
+      <c r="AD2" s="5"/>
+      <c r="AE2" s="5"/>
+      <c r="AF2" s="5"/>
+      <c r="AG2" s="5"/>
+      <c r="AH2" s="5"/>
+      <c r="AI2" s="5"/>
+      <c r="AJ2" s="5"/>
+      <c r="AK2" s="5"/>
+      <c r="AL2" s="5"/>
+      <c r="AM2" s="5"/>
+      <c r="AN2" s="5"/>
     </row>
     <row r="3" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="4"/>
+      <c r="G3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
+      <c r="J3" s="4"/>
+      <c r="K3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3" t="s">
+      <c r="L3" s="4"/>
+      <c r="M3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3" t="s">
+      <c r="N3" s="4"/>
+      <c r="O3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3" t="s">
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3" t="s">
+      <c r="R3" s="4"/>
+      <c r="S3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3" t="s">
+      <c r="T3" s="4"/>
+      <c r="U3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3" t="s">
+      <c r="V3" s="4"/>
+      <c r="W3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3" t="s">
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="3" t="s">
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3" t="s">
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AD3" s="3"/>
-      <c r="AE3" s="3" t="s">
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3" t="s">
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3" t="s">
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AJ3" s="3"/>
-      <c r="AK3" s="3" t="s">
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AL3" s="3"/>
-      <c r="AM3" s="3" t="s">
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AN3" s="3"/>
+      <c r="AN3" s="4"/>
     </row>
     <row r="4" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
+      <c r="F4" s="4"/>
+      <c r="G4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3" t="s">
+      <c r="H4" s="4"/>
+      <c r="I4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="4"/>
+      <c r="K4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3" t="s">
+      <c r="L4" s="4"/>
+      <c r="M4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3" t="s">
+      <c r="N4" s="4"/>
+      <c r="O4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3" t="s">
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3" t="s">
+      <c r="R4" s="4"/>
+      <c r="S4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3" t="s">
+      <c r="T4" s="4"/>
+      <c r="U4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3" t="s">
+      <c r="V4" s="4"/>
+      <c r="W4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3" t="s">
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3" t="s">
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="3" t="s">
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AD4" s="3"/>
-      <c r="AE4" s="3" t="s">
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="3" t="s">
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="AH4" s="3"/>
-      <c r="AI4" s="3" t="s">
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AJ4" s="3"/>
-      <c r="AK4" s="3" t="s">
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AL4" s="3"/>
-      <c r="AM4" s="3" t="s">
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AN4" s="3"/>
+      <c r="AN4" s="4"/>
     </row>
     <row r="5" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
@@ -18574,14 +19889,8 @@
       <c r="R22" t="s">
         <v>76</v>
       </c>
-      <c r="S22" t="s">
-        <v>45</v>
-      </c>
-      <c r="T22" t="s">
-        <v>45</v>
-      </c>
       <c r="U22" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="2:40" x14ac:dyDescent="0.3">
@@ -18636,14 +19945,8 @@
       <c r="R23" t="s">
         <v>75</v>
       </c>
-      <c r="S23" t="s">
-        <v>47</v>
-      </c>
-      <c r="T23" t="s">
-        <v>48</v>
-      </c>
       <c r="U23" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="2:40" x14ac:dyDescent="0.3">
@@ -18714,18 +20017,6 @@
         <f>AG9*100</f>
         <v>99.60703147712556</v>
       </c>
-      <c r="S24">
-        <f>AI9*100</f>
-        <v>0</v>
-      </c>
-      <c r="T24">
-        <f>AK9*100</f>
-        <v>0</v>
-      </c>
-      <c r="U24">
-        <f>AM9*100</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="25" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
@@ -18795,18 +20086,6 @@
         <f>AH9*100</f>
         <v>99.821700201624736</v>
       </c>
-      <c r="S25">
-        <f>AJ9*100</f>
-        <v>0</v>
-      </c>
-      <c r="T25">
-        <f>AL9*100</f>
-        <v>0</v>
-      </c>
-      <c r="U25">
-        <f>AN9*100</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="26" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
@@ -18876,22 +20155,14 @@
         <f>IFERROR(((AG6-AH6)/AG6)*100, 0)</f>
         <v>47.625052543085324</v>
       </c>
-      <c r="S26">
-        <f>IFERROR(((AI6-AJ6)/AI6)*100, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="T26">
-        <f>IFERROR(((AK6-AL6)/AK6)*100, 0)</f>
-        <v>0</v>
-      </c>
       <c r="U26">
-        <f>IFERROR(((AM6-AN6)/AM6)*100, 0)</f>
-        <v>0</v>
+        <f>SUM(C26:R26)/COLUMNS(C26:R26)</f>
+        <v>34.353165863987456</v>
       </c>
     </row>
     <row r="27" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C27">
         <f>C13</f>
@@ -18957,22 +20228,14 @@
         <f>AG13</f>
         <v>0.3030685161832703</v>
       </c>
-      <c r="S27">
-        <f>AI13</f>
-        <v>0</v>
-      </c>
-      <c r="T27">
-        <f>AK13</f>
-        <v>0</v>
-      </c>
       <c r="U27">
-        <f>AM13</f>
-        <v>0</v>
+        <f>SUM(C27:R27)/COLUMNS(C27:R27)</f>
+        <v>0.39307622869439407</v>
       </c>
     </row>
     <row r="28" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="C28">
         <f>D13</f>
@@ -19038,223 +20301,215 @@
         <f>AH13</f>
         <v>0.5786516853932584</v>
       </c>
-      <c r="S28">
-        <f>AJ13</f>
-        <v>0</v>
-      </c>
-      <c r="T28">
-        <f>AL13</f>
-        <v>0</v>
-      </c>
       <c r="U28">
-        <f>AN13</f>
-        <v>0</v>
+        <f>SUM(C28:R28)/COLUMNS(C28:R28)</f>
+        <v>0.61038406266350664</v>
       </c>
     </row>
     <row r="84" spans="2:40" x14ac:dyDescent="0.3">
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C84" s="5"/>
-      <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
-      <c r="I84" s="5"/>
-      <c r="J84" s="5"/>
-      <c r="K84" s="5"/>
-      <c r="L84" s="5"/>
-      <c r="M84" s="5"/>
-      <c r="N84" s="5"/>
-      <c r="O84" s="5"/>
-      <c r="P84" s="5"/>
-      <c r="Q84" s="5"/>
-      <c r="R84" s="5"/>
-      <c r="S84" s="5"/>
-      <c r="T84" s="5"/>
-      <c r="U84" s="5"/>
-      <c r="V84" s="5"/>
-      <c r="W84" s="5"/>
-      <c r="X84" s="5"/>
-      <c r="Y84" s="5"/>
-      <c r="Z84" s="5"/>
-      <c r="AA84" s="5"/>
-      <c r="AB84" s="5"/>
-      <c r="AC84" s="5"/>
-      <c r="AD84" s="5"/>
-      <c r="AE84" s="5"/>
-      <c r="AF84" s="5"/>
-      <c r="AG84" s="5"/>
-      <c r="AH84" s="5"/>
-      <c r="AI84" s="5"/>
-      <c r="AJ84" s="5"/>
-      <c r="AK84" s="5"/>
-      <c r="AL84" s="5"/>
-      <c r="AM84" s="5"/>
-      <c r="AN84" s="5"/>
+      <c r="C84" s="6"/>
+      <c r="D84" s="6"/>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
+      <c r="H84" s="6"/>
+      <c r="I84" s="6"/>
+      <c r="J84" s="6"/>
+      <c r="K84" s="6"/>
+      <c r="L84" s="6"/>
+      <c r="M84" s="6"/>
+      <c r="N84" s="6"/>
+      <c r="O84" s="6"/>
+      <c r="P84" s="6"/>
+      <c r="Q84" s="6"/>
+      <c r="R84" s="6"/>
+      <c r="S84" s="6"/>
+      <c r="T84" s="6"/>
+      <c r="U84" s="6"/>
+      <c r="V84" s="6"/>
+      <c r="W84" s="6"/>
+      <c r="X84" s="6"/>
+      <c r="Y84" s="6"/>
+      <c r="Z84" s="6"/>
+      <c r="AA84" s="6"/>
+      <c r="AB84" s="6"/>
+      <c r="AC84" s="6"/>
+      <c r="AD84" s="6"/>
+      <c r="AE84" s="6"/>
+      <c r="AF84" s="6"/>
+      <c r="AG84" s="6"/>
+      <c r="AH84" s="6"/>
+      <c r="AI84" s="6"/>
+      <c r="AJ84" s="6"/>
+      <c r="AK84" s="6"/>
+      <c r="AL84" s="6"/>
+      <c r="AM84" s="6"/>
+      <c r="AN84" s="6"/>
     </row>
     <row r="85" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>27</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="C85" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3" t="s">
+      <c r="D85" s="4"/>
+      <c r="E85" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F85" s="3"/>
-      <c r="G85" s="3" t="s">
+      <c r="F85" s="4"/>
+      <c r="G85" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H85" s="3"/>
-      <c r="I85" s="3" t="s">
+      <c r="H85" s="4"/>
+      <c r="I85" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J85" s="3"/>
-      <c r="K85" s="3" t="s">
+      <c r="J85" s="4"/>
+      <c r="K85" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="L85" s="3"/>
-      <c r="M85" s="3" t="s">
+      <c r="L85" s="4"/>
+      <c r="M85" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N85" s="3"/>
-      <c r="O85" s="3" t="s">
+      <c r="N85" s="4"/>
+      <c r="O85" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="P85" s="3"/>
-      <c r="Q85" s="3" t="s">
+      <c r="P85" s="4"/>
+      <c r="Q85" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R85" s="3"/>
-      <c r="S85" s="3" t="s">
+      <c r="R85" s="4"/>
+      <c r="S85" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="T85" s="3"/>
-      <c r="U85" s="3" t="s">
+      <c r="T85" s="4"/>
+      <c r="U85" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="V85" s="3"/>
-      <c r="W85" s="3" t="s">
+      <c r="V85" s="4"/>
+      <c r="W85" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="X85" s="3"/>
-      <c r="Y85" s="3" t="s">
+      <c r="X85" s="4"/>
+      <c r="Y85" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="Z85" s="3"/>
-      <c r="AA85" s="3" t="s">
+      <c r="Z85" s="4"/>
+      <c r="AA85" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AB85" s="3"/>
-      <c r="AC85" s="3" t="s">
+      <c r="AB85" s="4"/>
+      <c r="AC85" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AD85" s="3"/>
-      <c r="AE85" s="3" t="s">
+      <c r="AD85" s="4"/>
+      <c r="AE85" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AF85" s="3"/>
-      <c r="AG85" s="3" t="s">
+      <c r="AF85" s="4"/>
+      <c r="AG85" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="AH85" s="3"/>
-      <c r="AI85" s="3" t="s">
+      <c r="AH85" s="4"/>
+      <c r="AI85" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AJ85" s="3"/>
-      <c r="AK85" s="3" t="s">
+      <c r="AJ85" s="4"/>
+      <c r="AK85" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AL85" s="3"/>
-      <c r="AM85" s="3" t="s">
+      <c r="AL85" s="4"/>
+      <c r="AM85" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AN85" s="3"/>
+      <c r="AN85" s="4"/>
     </row>
     <row r="86" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>26</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3" t="s">
+      <c r="D86" s="4"/>
+      <c r="E86" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3" t="s">
+      <c r="F86" s="4"/>
+      <c r="G86" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3" t="s">
+      <c r="H86" s="4"/>
+      <c r="I86" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3" t="s">
+      <c r="J86" s="4"/>
+      <c r="K86" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3" t="s">
+      <c r="L86" s="4"/>
+      <c r="M86" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3" t="s">
+      <c r="N86" s="4"/>
+      <c r="O86" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3" t="s">
+      <c r="P86" s="4"/>
+      <c r="Q86" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3" t="s">
+      <c r="R86" s="4"/>
+      <c r="S86" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3" t="s">
+      <c r="T86" s="4"/>
+      <c r="U86" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V86" s="3"/>
-      <c r="W86" s="3" t="s">
+      <c r="V86" s="4"/>
+      <c r="W86" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="X86" s="3"/>
-      <c r="Y86" s="3" t="s">
+      <c r="X86" s="4"/>
+      <c r="Y86" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Z86" s="3"/>
-      <c r="AA86" s="3" t="s">
+      <c r="Z86" s="4"/>
+      <c r="AA86" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AB86" s="3"/>
-      <c r="AC86" s="3" t="s">
+      <c r="AB86" s="4"/>
+      <c r="AC86" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AD86" s="3"/>
-      <c r="AE86" s="3" t="s">
+      <c r="AD86" s="4"/>
+      <c r="AE86" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AF86" s="3"/>
-      <c r="AG86" s="3" t="s">
+      <c r="AF86" s="4"/>
+      <c r="AG86" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="AH86" s="3"/>
-      <c r="AI86" s="3" t="s">
+      <c r="AH86" s="4"/>
+      <c r="AI86" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AJ86" s="3"/>
-      <c r="AK86" s="3" t="s">
+      <c r="AJ86" s="4"/>
+      <c r="AK86" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AL86" s="3"/>
-      <c r="AM86" s="3" t="s">
+      <c r="AL86" s="4"/>
+      <c r="AM86" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AN86" s="3"/>
+      <c r="AN86" s="4"/>
     </row>
     <row r="87" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
@@ -21007,14 +22262,8 @@
       <c r="R104" t="s">
         <v>76</v>
       </c>
-      <c r="S104" t="s">
-        <v>45</v>
-      </c>
-      <c r="T104" t="s">
-        <v>45</v>
-      </c>
       <c r="U104" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="105" spans="2:40" x14ac:dyDescent="0.3">
@@ -21069,14 +22318,8 @@
       <c r="R105" t="s">
         <v>75</v>
       </c>
-      <c r="S105" t="s">
-        <v>47</v>
-      </c>
-      <c r="T105" t="s">
-        <v>48</v>
-      </c>
       <c r="U105" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
     </row>
     <row r="106" spans="2:40" x14ac:dyDescent="0.3">
@@ -21147,18 +22390,6 @@
         <f>AG91*100</f>
         <v>99.60703147712556</v>
       </c>
-      <c r="S106">
-        <f>AI91*100</f>
-        <v>0</v>
-      </c>
-      <c r="T106">
-        <f>AK91*100</f>
-        <v>0</v>
-      </c>
-      <c r="U106">
-        <f>AM91*100</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="107" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
@@ -21228,18 +22459,6 @@
         <f>AH91*100</f>
         <v>99.821700201624736</v>
       </c>
-      <c r="S107">
-        <f>AJ91*100</f>
-        <v>0</v>
-      </c>
-      <c r="T107">
-        <f>AL91*100</f>
-        <v>0</v>
-      </c>
-      <c r="U107">
-        <f>AN91*100</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="108" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
@@ -21309,22 +22528,14 @@
         <f>IFERROR(((AG88-AH88)/AG88)*100, 0)</f>
         <v>47.625052543085324</v>
       </c>
-      <c r="S108">
-        <f>IFERROR(((AI88-AJ88)/AI88)*100, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="T108">
-        <f>IFERROR(((AK88-AL88)/AK88)*100, 0)</f>
-        <v>0</v>
-      </c>
       <c r="U108">
-        <f>IFERROR(((AM88-AN88)/AM88)*100, 0)</f>
-        <v>0</v>
+        <f>SUM(C108:R108)/COLUMNS(C108:R108)</f>
+        <v>36.215861874989677</v>
       </c>
     </row>
     <row r="109" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C109">
         <f>C95</f>
@@ -21390,22 +22601,14 @@
         <f>AG95</f>
         <v>0.3030685161832703</v>
       </c>
-      <c r="S109">
-        <f>AI95</f>
-        <v>0</v>
-      </c>
-      <c r="T109">
-        <f>AK95</f>
-        <v>0</v>
-      </c>
       <c r="U109">
-        <f>AM95</f>
-        <v>0</v>
+        <f>SUM(C109:R109)/COLUMNS(C109:R109)</f>
+        <v>0.39307622869439407</v>
       </c>
     </row>
     <row r="110" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="C110">
         <f>D95</f>
@@ -21471,179 +22674,147 @@
         <f>AH95</f>
         <v>0.5786516853932584</v>
       </c>
-      <c r="S110">
-        <f>AJ95</f>
-        <v>0</v>
-      </c>
-      <c r="T110">
-        <f>AL95</f>
-        <v>0</v>
-      </c>
       <c r="U110">
-        <f>AN95</f>
-        <v>0</v>
+        <f>SUM(C110:R110)/COLUMNS(C110:R110)</f>
+        <v>0.62454697134445358</v>
       </c>
     </row>
     <row r="156" spans="2:40" x14ac:dyDescent="0.3">
-      <c r="B156" s="6" t="s">
+      <c r="B156" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C156" s="6"/>
-      <c r="D156" s="6"/>
-      <c r="E156" s="6"/>
-      <c r="F156" s="6"/>
-      <c r="G156" s="6"/>
-      <c r="H156" s="6"/>
-      <c r="I156" s="6"/>
-      <c r="J156" s="6"/>
-      <c r="K156" s="6"/>
-      <c r="L156" s="6"/>
-      <c r="M156" s="6"/>
-      <c r="N156" s="6"/>
-      <c r="O156" s="6"/>
-      <c r="P156" s="6"/>
-      <c r="Q156" s="7"/>
-      <c r="R156" s="7"/>
-      <c r="S156" s="7"/>
-      <c r="T156" s="7"/>
-      <c r="U156" s="7"/>
-      <c r="V156" s="7"/>
-      <c r="W156" s="7"/>
-      <c r="X156" s="7"/>
-      <c r="Y156" s="7"/>
-      <c r="Z156" s="7"/>
-      <c r="AA156" s="7"/>
-      <c r="AB156" s="7"/>
-      <c r="AC156" s="7"/>
-      <c r="AD156" s="7"/>
-      <c r="AE156" s="7"/>
-      <c r="AF156" s="7"/>
-      <c r="AG156" s="7"/>
-      <c r="AH156" s="7"/>
-      <c r="AI156" s="7"/>
-      <c r="AJ156" s="7"/>
-      <c r="AK156" s="7"/>
-      <c r="AL156" s="7"/>
-      <c r="AM156" s="7"/>
-      <c r="AN156" s="7"/>
+      <c r="C156" s="7"/>
+      <c r="D156" s="7"/>
+      <c r="E156" s="7"/>
+      <c r="F156" s="7"/>
+      <c r="G156" s="7"/>
+      <c r="H156" s="7"/>
+      <c r="I156" s="7"/>
+      <c r="J156" s="7"/>
+      <c r="K156" s="7"/>
+      <c r="L156" s="7"/>
+      <c r="M156" s="7"/>
+      <c r="N156" s="7"/>
+      <c r="O156" s="7"/>
+      <c r="P156" s="7"/>
     </row>
     <row r="157" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>27</v>
       </c>
-      <c r="C157" s="3" t="s">
+      <c r="C157" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D157" s="3"/>
-      <c r="E157" s="3" t="s">
+      <c r="D157" s="4"/>
+      <c r="E157" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F157" s="3"/>
-      <c r="G157" s="3" t="s">
+      <c r="F157" s="4"/>
+      <c r="G157" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H157" s="3"/>
-      <c r="I157" s="3" t="s">
+      <c r="H157" s="4"/>
+      <c r="I157" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="J157" s="3"/>
-      <c r="K157" s="3" t="s">
+      <c r="J157" s="4"/>
+      <c r="K157" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="L157" s="3"/>
-      <c r="M157" s="3" t="s">
+      <c r="L157" s="4"/>
+      <c r="M157" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="N157" s="3"/>
-      <c r="O157" s="3" t="s">
+      <c r="N157" s="4"/>
+      <c r="O157" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="P157" s="3"/>
+      <c r="P157" s="4"/>
       <c r="Q157" s="2" t="s">
         <v>66</v>
       </c>
       <c r="R157" s="2"/>
-      <c r="S157" s="3"/>
-      <c r="T157" s="3"/>
-      <c r="U157" s="3"/>
-      <c r="V157" s="3"/>
-      <c r="W157" s="3"/>
-      <c r="X157" s="3"/>
-      <c r="Y157" s="3"/>
-      <c r="Z157" s="3"/>
-      <c r="AA157" s="3"/>
-      <c r="AB157" s="3"/>
-      <c r="AC157" s="3"/>
-      <c r="AD157" s="3"/>
-      <c r="AE157" s="3"/>
-      <c r="AF157" s="3"/>
-      <c r="AG157" s="3"/>
-      <c r="AH157" s="3"/>
-      <c r="AI157" s="3"/>
-      <c r="AJ157" s="3"/>
-      <c r="AK157" s="3"/>
-      <c r="AL157" s="3"/>
-      <c r="AM157" s="3"/>
-      <c r="AN157" s="3"/>
+      <c r="S157" s="4"/>
+      <c r="T157" s="4"/>
+      <c r="U157" s="4"/>
+      <c r="V157" s="4"/>
+      <c r="W157" s="4"/>
+      <c r="X157" s="4"/>
+      <c r="Y157" s="4"/>
+      <c r="Z157" s="4"/>
+      <c r="AA157" s="4"/>
+      <c r="AB157" s="4"/>
+      <c r="AC157" s="4"/>
+      <c r="AD157" s="4"/>
+      <c r="AE157" s="4"/>
+      <c r="AF157" s="4"/>
+      <c r="AG157" s="4"/>
+      <c r="AH157" s="4"/>
+      <c r="AI157" s="4"/>
+      <c r="AJ157" s="4"/>
+      <c r="AK157" s="4"/>
+      <c r="AL157" s="4"/>
+      <c r="AM157" s="4"/>
+      <c r="AN157" s="4"/>
     </row>
     <row r="158" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>26</v>
       </c>
-      <c r="C158" s="3" t="s">
+      <c r="C158" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D158" s="3"/>
-      <c r="E158" s="3" t="s">
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F158" s="3"/>
-      <c r="G158" s="3" t="s">
+      <c r="F158" s="4"/>
+      <c r="G158" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H158" s="3"/>
-      <c r="I158" s="3" t="s">
+      <c r="H158" s="4"/>
+      <c r="I158" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="J158" s="3"/>
-      <c r="K158" s="3" t="s">
+      <c r="J158" s="4"/>
+      <c r="K158" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="L158" s="3"/>
-      <c r="M158" s="3" t="s">
+      <c r="L158" s="4"/>
+      <c r="M158" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="N158" s="3"/>
-      <c r="O158" s="3" t="s">
+      <c r="N158" s="4"/>
+      <c r="O158" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="P158" s="3"/>
+      <c r="P158" s="4"/>
       <c r="Q158" s="2" t="s">
         <v>72</v>
       </c>
       <c r="R158" s="2"/>
-      <c r="S158" s="3"/>
-      <c r="T158" s="3"/>
-      <c r="U158" s="3"/>
-      <c r="V158" s="3"/>
-      <c r="W158" s="3"/>
-      <c r="X158" s="3"/>
-      <c r="Y158" s="3"/>
-      <c r="Z158" s="3"/>
-      <c r="AA158" s="3"/>
-      <c r="AB158" s="3"/>
-      <c r="AC158" s="3"/>
-      <c r="AD158" s="3"/>
-      <c r="AE158" s="3"/>
-      <c r="AF158" s="3"/>
-      <c r="AG158" s="3"/>
-      <c r="AH158" s="3"/>
-      <c r="AI158" s="3"/>
-      <c r="AJ158" s="3"/>
-      <c r="AK158" s="3"/>
-      <c r="AL158" s="3"/>
-      <c r="AM158" s="3"/>
-      <c r="AN158" s="3"/>
+      <c r="S158" s="4"/>
+      <c r="T158" s="4"/>
+      <c r="U158" s="4"/>
+      <c r="V158" s="4"/>
+      <c r="W158" s="4"/>
+      <c r="X158" s="4"/>
+      <c r="Y158" s="4"/>
+      <c r="Z158" s="4"/>
+      <c r="AA158" s="4"/>
+      <c r="AB158" s="4"/>
+      <c r="AC158" s="4"/>
+      <c r="AD158" s="4"/>
+      <c r="AE158" s="4"/>
+      <c r="AF158" s="4"/>
+      <c r="AG158" s="4"/>
+      <c r="AH158" s="4"/>
+      <c r="AI158" s="4"/>
+      <c r="AJ158" s="4"/>
+      <c r="AK158" s="4"/>
+      <c r="AL158" s="4"/>
+      <c r="AM158" s="4"/>
+      <c r="AN158" s="4"/>
     </row>
     <row r="159" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
@@ -22792,11 +23963,16 @@
       </c>
     </row>
     <row r="187" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B187" s="8" t="s">
+      <c r="B187" s="3" t="s">
         <v>74</v>
       </c>
       <c r="C187" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="188" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C188" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -22825,18 +24001,6 @@
     <mergeCell ref="W158:X158"/>
     <mergeCell ref="Y158:Z158"/>
     <mergeCell ref="C157:D157"/>
-    <mergeCell ref="E157:F157"/>
-    <mergeCell ref="G157:H157"/>
-    <mergeCell ref="I157:J157"/>
-    <mergeCell ref="K157:L157"/>
-    <mergeCell ref="M157:N157"/>
-    <mergeCell ref="O157:P157"/>
-    <mergeCell ref="S157:T157"/>
-    <mergeCell ref="U157:V157"/>
-    <mergeCell ref="W157:X157"/>
-    <mergeCell ref="Y157:Z157"/>
-    <mergeCell ref="AA157:AB157"/>
-    <mergeCell ref="AC157:AD157"/>
     <mergeCell ref="AE157:AF157"/>
     <mergeCell ref="AM4:AN4"/>
     <mergeCell ref="AA4:AB4"/>
@@ -22845,17 +24009,37 @@
     <mergeCell ref="AG4:AH4"/>
     <mergeCell ref="AI4:AJ4"/>
     <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B84:AN84"/>
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="E85:F85"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="I85:J85"/>
+    <mergeCell ref="K85:L85"/>
+    <mergeCell ref="M85:N85"/>
+    <mergeCell ref="O85:P85"/>
+    <mergeCell ref="Q85:R85"/>
+    <mergeCell ref="S85:T85"/>
+    <mergeCell ref="U85:V85"/>
+    <mergeCell ref="W85:X85"/>
+    <mergeCell ref="Y85:Z85"/>
+    <mergeCell ref="E157:F157"/>
+    <mergeCell ref="G157:H157"/>
+    <mergeCell ref="I157:J157"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:X3"/>
     <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="Y157:Z157"/>
+    <mergeCell ref="AA157:AB157"/>
+    <mergeCell ref="AC157:AD157"/>
+    <mergeCell ref="K157:L157"/>
+    <mergeCell ref="M157:N157"/>
+    <mergeCell ref="O157:P157"/>
+    <mergeCell ref="S157:T157"/>
+    <mergeCell ref="U157:V157"/>
+    <mergeCell ref="W157:X157"/>
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="S4:T4"/>
@@ -22877,26 +24061,19 @@
     <mergeCell ref="AM3:AN3"/>
     <mergeCell ref="AC3:AD3"/>
     <mergeCell ref="AE3:AF3"/>
-    <mergeCell ref="B84:AN84"/>
-    <mergeCell ref="C85:D85"/>
-    <mergeCell ref="E85:F85"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="I85:J85"/>
-    <mergeCell ref="K85:L85"/>
-    <mergeCell ref="M85:N85"/>
-    <mergeCell ref="O85:P85"/>
-    <mergeCell ref="Q85:R85"/>
-    <mergeCell ref="S85:T85"/>
-    <mergeCell ref="U85:V85"/>
-    <mergeCell ref="W85:X85"/>
-    <mergeCell ref="Y85:Z85"/>
-    <mergeCell ref="AA85:AB85"/>
-    <mergeCell ref="AC85:AD85"/>
-    <mergeCell ref="AE85:AF85"/>
-    <mergeCell ref="AG85:AH85"/>
-    <mergeCell ref="AI85:AJ85"/>
-    <mergeCell ref="AK85:AL85"/>
-    <mergeCell ref="AM85:AN85"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="U86:V86"/>
+    <mergeCell ref="W86:X86"/>
+    <mergeCell ref="Y86:Z86"/>
+    <mergeCell ref="AK86:AL86"/>
+    <mergeCell ref="AM86:AN86"/>
+    <mergeCell ref="AA86:AB86"/>
+    <mergeCell ref="AC86:AD86"/>
+    <mergeCell ref="AE86:AF86"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="C86:D86"/>
     <mergeCell ref="E86:F86"/>
     <mergeCell ref="G86:H86"/>
@@ -22906,16 +24083,15 @@
     <mergeCell ref="O86:P86"/>
     <mergeCell ref="Q86:R86"/>
     <mergeCell ref="S86:T86"/>
-    <mergeCell ref="U86:V86"/>
-    <mergeCell ref="W86:X86"/>
-    <mergeCell ref="Y86:Z86"/>
-    <mergeCell ref="AK86:AL86"/>
-    <mergeCell ref="AM86:AN86"/>
-    <mergeCell ref="AA86:AB86"/>
-    <mergeCell ref="AC86:AD86"/>
-    <mergeCell ref="AE86:AF86"/>
     <mergeCell ref="AG86:AH86"/>
     <mergeCell ref="AI86:AJ86"/>
+    <mergeCell ref="AA85:AB85"/>
+    <mergeCell ref="AC85:AD85"/>
+    <mergeCell ref="AE85:AF85"/>
+    <mergeCell ref="AG85:AH85"/>
+    <mergeCell ref="AI85:AJ85"/>
+    <mergeCell ref="AK85:AL85"/>
+    <mergeCell ref="AM85:AN85"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>